<commit_message>
Fixed crucial spelling mistakes - future warning: Mapping function is case sensitivy and only works with lowercase letters. Expects ONLY - and _. No spaces allowed
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/Zwischenstände/CAES2024_Datenbank/after_conversion_caes2014_mapped_readable.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/Zwischenstände/CAES2024_Datenbank/after_conversion_caes2014_mapped_readable.xlsx
@@ -638,14 +638,13 @@
     <col min="7" max="7" width="22.7109375" customWidth="1"/>
     <col min="8" max="8" width="18.7109375" customWidth="1"/>
     <col min="9" max="9" width="38.7109375" customWidth="1"/>
-    <col min="10" max="10" width="5.7109375" customWidth="1"/>
+    <col min="10" max="10" width="6.7109375" customWidth="1"/>
     <col min="11" max="11" width="23.7109375" customWidth="1"/>
     <col min="12" max="12" width="34.7109375" customWidth="1"/>
     <col min="13" max="13" width="14.7109375" customWidth="1"/>
     <col min="14" max="14" width="20.7109375" customWidth="1"/>
     <col min="15" max="15" width="23.7109375" customWidth="1"/>
-    <col min="16" max="21" width="20.7109375" customWidth="1"/>
-    <col min="22" max="22" width="14.7109375" customWidth="1"/>
+    <col min="16" max="22" width="20.7109375" customWidth="1"/>
     <col min="23" max="23" width="15.7109375" customWidth="1"/>
     <col min="24" max="25" width="14.7109375" customWidth="1"/>
     <col min="26" max="26" width="20.7109375" customWidth="1"/>
@@ -763,8 +762,11 @@
       <c r="H2">
         <v>48.2</v>
       </c>
+      <c r="J2">
+        <v>6.32</v>
+      </c>
       <c r="L2">
-        <v>173.4775697006366</v>
+        <v>173.5399527182125</v>
       </c>
       <c r="N2">
         <v>66.98631900129141</v>
@@ -789,6 +791,9 @@
       </c>
       <c r="U2">
         <v>5.268771276500512</v>
+      </c>
+      <c r="V2">
+        <v>62.38301757589591</v>
       </c>
       <c r="Z2">
         <v>210.5484787872408</v>
@@ -813,8 +818,11 @@
       <c r="H3">
         <v>56.1</v>
       </c>
+      <c r="J3">
+        <v>7.17</v>
+      </c>
       <c r="L3">
-        <v>7.004147355459007</v>
+        <v>7.010960868355606</v>
       </c>
       <c r="N3">
         <v>1.087440243527458</v>
@@ -839,6 +847,9 @@
       </c>
       <c r="U3">
         <v>0.3376105866495474</v>
+      </c>
+      <c r="V3">
+        <v>6.813512896598949</v>
       </c>
       <c r="Z3">
         <v>242.1307506053269</v>
@@ -863,8 +874,11 @@
       <c r="H4">
         <v>52.3</v>
       </c>
+      <c r="J4">
+        <v>7.21</v>
+      </c>
       <c r="L4">
-        <v>7.502501946532076</v>
+        <v>7.509475240300623</v>
       </c>
       <c r="N4">
         <v>1.217933072750753</v>
@@ -889,6 +903,9 @@
       </c>
       <c r="U4">
         <v>0.3452835545279462</v>
+      </c>
+      <c r="V4">
+        <v>6.973293768545994</v>
       </c>
       <c r="Z4">
         <v>247.3944625750079</v>
@@ -913,8 +930,11 @@
       <c r="H5">
         <v>44</v>
       </c>
+      <c r="J5">
+        <v>7.2</v>
+      </c>
       <c r="L5">
-        <v>10.53010726880455</v>
+        <v>10.54348321037041</v>
       </c>
       <c r="N5">
         <v>0.2174880487054915</v>
@@ -939,6 +959,9 @@
       </c>
       <c r="U5">
         <v>0.115094518175982</v>
+      </c>
+      <c r="V5">
+        <v>13.37594156585254</v>
       </c>
       <c r="Z5">
         <v>78.95567954521528</v>
@@ -966,8 +989,11 @@
       <c r="H6">
         <v>31.4</v>
       </c>
+      <c r="J6">
+        <v>8.73</v>
+      </c>
       <c r="L6">
-        <v>2.696471744017176</v>
+        <v>2.6965288086143</v>
       </c>
       <c r="N6">
         <v>1.435421121456244</v>
@@ -992,6 +1018,9 @@
       </c>
       <c r="U6">
         <v>0.0230189036351964</v>
+      </c>
+      <c r="V6">
+        <v>0.0570645971239443</v>
       </c>
       <c r="Z6">
         <v>110.5379513633014</v>
@@ -1016,8 +1045,11 @@
       <c r="H7">
         <v>50.5</v>
       </c>
+      <c r="J7">
+        <v>7.03</v>
+      </c>
       <c r="L7">
-        <v>10.33282162867493</v>
+        <v>10.34345846957883</v>
       </c>
       <c r="N7">
         <v>2.696851803948096</v>
@@ -1042,6 +1074,9 @@
       </c>
       <c r="U7">
         <v>0.5754725908799103</v>
+      </c>
+      <c r="V7">
+        <v>10.63684090390322</v>
       </c>
       <c r="Z7">
         <v>84.21939151489632</v>
@@ -1069,8 +1104,11 @@
       <c r="H8">
         <v>36.3</v>
       </c>
+      <c r="J8">
+        <v>7.09</v>
+      </c>
       <c r="L8">
-        <v>9.90425299070561</v>
+        <v>9.912504531449732</v>
       </c>
       <c r="N8">
         <v>1.478918731197343</v>
@@ -1095,6 +1133,9 @@
       </c>
       <c r="U8">
         <v>0.2404196601898292</v>
+      </c>
+      <c r="V8">
+        <v>8.251540744122345</v>
       </c>
       <c r="Z8">
         <v>36.84598378776712</v>
@@ -1122,8 +1163,11 @@
       <c r="H9">
         <v>24.7</v>
       </c>
+      <c r="J9">
+        <v>9.470000000000001</v>
+      </c>
       <c r="L9">
-        <v>9.165468661159901</v>
+        <v>9.165719745387246</v>
       </c>
       <c r="N9">
         <v>4.91522990074411</v>
@@ -1148,6 +1192,9 @@
       </c>
       <c r="U9">
         <v>0.1074215502975832</v>
+      </c>
+      <c r="V9">
+        <v>0.2510842273453549</v>
       </c>
       <c r="Z9">
         <v>642.1728603010843</v>
@@ -1175,8 +1222,11 @@
       <c r="H10">
         <v>34.5</v>
       </c>
+      <c r="J10">
+        <v>7.98</v>
+      </c>
       <c r="L10">
-        <v>6.552787235806358</v>
+        <v>6.554567651236625</v>
       </c>
       <c r="N10">
         <v>2.522861364983702</v>
@@ -1201,6 +1251,9 @@
       </c>
       <c r="U10">
         <v>0.1969395088789026</v>
+      </c>
+      <c r="V10">
+        <v>1.780415430267063</v>
       </c>
       <c r="Z10">
         <v>115.8016633329824</v>
@@ -1228,8 +1281,11 @@
       <c r="H11">
         <v>34.4</v>
       </c>
+      <c r="J11">
+        <v>7.96</v>
+      </c>
       <c r="L11">
-        <v>6.190859106790139</v>
+        <v>6.192879193528326</v>
       </c>
       <c r="N11">
         <v>2.435866145501505</v>
@@ -1254,6 +1310,9 @@
       </c>
       <c r="U11">
         <v>0.2046124767573014</v>
+      </c>
+      <c r="V11">
+        <v>2.020086738187628</v>
       </c>
       <c r="Z11">
         <v>131.5927992420255</v>
@@ -1278,8 +1337,11 @@
       <c r="H12">
         <v>58.4</v>
       </c>
+      <c r="J12">
+        <v>9.529999999999999</v>
+      </c>
       <c r="L12">
-        <v>9.324216478632884</v>
+        <v>9.32422789155231</v>
       </c>
       <c r="N12">
         <v>5.567694046860584</v>
@@ -1304,6 +1366,9 @@
       </c>
       <c r="U12">
         <v>0.048595463229859</v>
+      </c>
+      <c r="V12">
+        <v>0.0114129194247888</v>
       </c>
       <c r="Z12">
         <v>1179.071481208548</v>
@@ -1331,8 +1396,11 @@
       <c r="H13">
         <v>37.5</v>
       </c>
+      <c r="J13">
+        <v>8.59</v>
+      </c>
       <c r="L13">
-        <v>11.69502292499311</v>
+        <v>11.69574193891687</v>
       </c>
       <c r="N13">
         <v>6.481143851423648</v>
@@ -1357,6 +1425,9 @@
       </c>
       <c r="U13">
         <v>0.0358071834325277</v>
+      </c>
+      <c r="V13">
+        <v>0.7190139237616983</v>
       </c>
       <c r="Z13">
         <v>126.3290872723444</v>
@@ -1381,8 +1452,11 @@
       <c r="H14">
         <v>36.2</v>
       </c>
+      <c r="J14">
+        <v>8.65</v>
+      </c>
       <c r="L14">
-        <v>11.68687731051054</v>
+        <v>11.68761915027315</v>
       </c>
       <c r="N14">
         <v>6.394148631941452</v>
@@ -1407,6 +1481,9 @@
       </c>
       <c r="U14">
         <v>0.048595463229859</v>
+      </c>
+      <c r="V14">
+        <v>0.741839762611276</v>
       </c>
       <c r="Z14">
         <v>126.3290872723444</v>
@@ -1434,8 +1511,11 @@
       <c r="H15">
         <v>38.1</v>
       </c>
+      <c r="J15">
+        <v>8.789999999999999</v>
+      </c>
       <c r="L15">
-        <v>7.770952248676309</v>
+        <v>7.771169094145381</v>
       </c>
       <c r="N15">
         <v>4.13227292540434</v>
@@ -1460,6 +1540,9 @@
       </c>
       <c r="U15">
         <v>0.0844026466623868</v>
+      </c>
+      <c r="V15">
+        <v>0.2168454690709883</v>
       </c>
       <c r="Z15">
         <v>505.3163490893778</v>
@@ -1484,8 +1567,11 @@
       <c r="H16">
         <v>20.9</v>
       </c>
+      <c r="J16">
+        <v>6.7</v>
+      </c>
       <c r="L16">
-        <v>13.41982456201163</v>
+        <v>13.42337186642729</v>
       </c>
       <c r="N16">
         <v>4.204596401120864</v>
@@ -1510,6 +1596,9 @@
       </c>
       <c r="U16">
         <v>0.4084346378231278</v>
+      </c>
+      <c r="V16">
+        <v>3.547304415658526</v>
       </c>
       <c r="Z16">
         <v>19.85998526160649</v>
@@ -1534,8 +1623,11 @@
       <c r="H17">
         <v>27.7</v>
       </c>
+      <c r="J17">
+        <v>6.94</v>
+      </c>
       <c r="L17">
-        <v>13.43038996411485</v>
+        <v>13.43316481844377</v>
       </c>
       <c r="N17">
         <v>3.903797380478247</v>
@@ -1560,6 +1652,9 @@
       </c>
       <c r="U17">
         <v>0.4033628060555062</v>
+      </c>
+      <c r="V17">
+        <v>2.774854328920338</v>
       </c>
       <c r="Z17">
         <v>14.06463838298768</v>
@@ -1584,8 +1679,11 @@
       <c r="H18">
         <v>26.8</v>
       </c>
+      <c r="J18">
+        <v>6.64</v>
+      </c>
       <c r="L18">
-        <v>18.52989578583409</v>
+        <v>18.53451418857775</v>
       </c>
       <c r="N18">
         <v>5.412294486299537</v>
@@ -1610,6 +1708,9 @@
       </c>
       <c r="U18">
         <v>0.4422468496072719</v>
+      </c>
+      <c r="V18">
+        <v>4.618402743665829</v>
       </c>
       <c r="Z18">
         <v>11.91704389935783</v>
@@ -1634,8 +1735,11 @@
       <c r="H19">
         <v>25.1</v>
       </c>
+      <c r="J19">
+        <v>6.77</v>
+      </c>
       <c r="L19">
-        <v>18.07812593914251</v>
+        <v>18.08302941785855</v>
       </c>
       <c r="N19">
         <v>5.316852031005618</v>
@@ -1660,6 +1764,9 @@
       </c>
       <c r="U19">
         <v>0.428138819334856</v>
+      </c>
+      <c r="V19">
+        <v>4.903478716046565</v>
       </c>
       <c r="Z19">
         <v>13.43299294662596</v>
@@ -1684,6 +1791,9 @@
       <c r="H20">
         <v>48.6</v>
       </c>
+      <c r="J20">
+        <v>6.31</v>
+      </c>
       <c r="L20">
         <v>14.75003605564369</v>
       </c>
@@ -1710,8 +1820,11 @@
       <c r="H21">
         <v>59.7</v>
       </c>
+      <c r="J21">
+        <v>7.05</v>
+      </c>
       <c r="L21">
-        <v>35.82082860627492</v>
+        <v>35.8382592345219</v>
       </c>
       <c r="N21">
         <v>24.69434555867004</v>
@@ -1733,6 +1846,9 @@
       </c>
       <c r="U21">
         <v>1.020358941437352</v>
+      </c>
+      <c r="V21">
+        <v>17.43062824697558</v>
       </c>
       <c r="Z21">
         <v>115.6963890935888</v>
@@ -1757,8 +1873,11 @@
       <c r="H22">
         <v>47.9</v>
       </c>
+      <c r="J22">
+        <v>6.92</v>
+      </c>
       <c r="L22">
-        <v>31.61343672170225</v>
+        <v>31.62740982383646</v>
       </c>
       <c r="N22">
         <v>18.19169640199517</v>
@@ -1780,6 +1899,9 @@
       </c>
       <c r="U22">
         <v>0.9690446899225796</v>
+      </c>
+      <c r="V22">
+        <v>13.97310213421593</v>
       </c>
       <c r="Z22">
         <v>244.1309611538056</v>
@@ -1804,8 +1926,11 @@
       <c r="H23">
         <v>48</v>
       </c>
+      <c r="J23">
+        <v>6.3</v>
+      </c>
       <c r="L23">
-        <v>126.6560297908685</v>
+        <v>126.7123079268763</v>
       </c>
       <c r="N23">
         <v>54.72829522558492</v>
@@ -1827,6 +1952,9 @@
       </c>
       <c r="U23">
         <v>3.843724663220651</v>
+      </c>
+      <c r="V23">
+        <v>56.27813600776079</v>
       </c>
       <c r="Z23">
         <v>318.1913885672176</v>
@@ -1851,8 +1979,11 @@
       <c r="H24">
         <v>48.3</v>
       </c>
+      <c r="J24">
+        <v>7.07</v>
+      </c>
       <c r="L24">
-        <v>50.19677584314741</v>
+        <v>50.21290334692509</v>
       </c>
       <c r="N24">
         <v>23.5995582687238</v>
@@ -1874,6 +2005,9 @@
       </c>
       <c r="U24">
         <v>0.9929076200244</v>
+      </c>
+      <c r="V24">
+        <v>16.12750377767633</v>
       </c>
       <c r="Z24">
         <v>376.4133066638593</v>
@@ -1898,8 +2032,11 @@
       <c r="H25">
         <v>32.7</v>
       </c>
+      <c r="J25">
+        <v>7.23</v>
+      </c>
       <c r="L25">
-        <v>17.93025620344883</v>
+        <v>17.954396415615</v>
       </c>
       <c r="N25">
         <v>5.482060028528343</v>
@@ -1924,6 +2061,9 @@
       </c>
       <c r="U25">
         <v>0.2935089249404705</v>
+      </c>
+      <c r="V25">
+        <v>24.14021216617211</v>
       </c>
       <c r="Z25">
         <v>26.4290977997684</v>
@@ -1948,8 +2088,11 @@
       <c r="H26">
         <v>54.7</v>
       </c>
+      <c r="J26">
+        <v>9.210000000000001</v>
+      </c>
       <c r="L26">
-        <v>13.59524702853911</v>
+        <v>13.5954275600326</v>
       </c>
       <c r="N26">
         <v>7.133889962095748</v>
@@ -1974,6 +2117,9 @@
       </c>
       <c r="U26">
         <v>0.0636165766798044</v>
+      </c>
+      <c r="V26">
+        <v>0.1805314934946359</v>
       </c>
       <c r="Z26">
         <v>352.5792188651437</v>
@@ -1998,8 +2144,11 @@
       <c r="H27">
         <v>44.7</v>
       </c>
+      <c r="J27">
+        <v>8.119999999999999</v>
+      </c>
       <c r="L27">
-        <v>59.43540772017607</v>
+        <v>59.45380732686404</v>
       </c>
       <c r="N27">
         <v>27.03231046819131</v>
@@ -2024,6 +2173,9 @@
       </c>
       <c r="U27">
         <v>0.6354879879687864</v>
+      </c>
+      <c r="V27">
+        <v>18.39960668797078</v>
       </c>
       <c r="Z27">
         <v>370.7811348563006</v>
@@ -2048,8 +2200,11 @@
       <c r="H28">
         <v>40.9</v>
       </c>
+      <c r="J28">
+        <v>7.72</v>
+      </c>
       <c r="L28">
-        <v>54.3713577494528</v>
+        <v>54.38896588154593</v>
       </c>
       <c r="N28">
         <v>26.02318118985885</v>
@@ -2074,6 +2229,9 @@
       </c>
       <c r="U28">
         <v>0.578268108843607</v>
+      </c>
+      <c r="V28">
+        <v>17.60813209312942</v>
       </c>
       <c r="Z28">
         <v>306.3743551952837</v>
@@ -2098,8 +2256,11 @@
       <c r="H29">
         <v>26</v>
       </c>
+      <c r="J29">
+        <v>8.27</v>
+      </c>
       <c r="L29">
-        <v>105.1530333881277</v>
+        <v>105.1886070966304</v>
       </c>
       <c r="N29">
         <v>51.62804097770621</v>
@@ -2124,6 +2285,9 @@
       </c>
       <c r="U29">
         <v>0.917692073568416</v>
+      </c>
+      <c r="V29">
+        <v>35.57370850262497</v>
       </c>
       <c r="Z29">
         <v>319.5810085272133</v>
@@ -2148,8 +2312,11 @@
       <c r="H30">
         <v>38.1</v>
       </c>
+      <c r="J30">
+        <v>7.25</v>
+      </c>
       <c r="L30">
-        <v>8.49263614046418</v>
+        <v>8.497765210273585</v>
       </c>
       <c r="N30">
         <v>1.868314941746479</v>
@@ -2174,6 +2341,9 @@
       </c>
       <c r="U30">
         <v>0.216244696060954</v>
+      </c>
+      <c r="V30">
+        <v>5.129069809404246</v>
       </c>
       <c r="Z30">
         <v>97.42078113485628</v>
@@ -2198,8 +2368,11 @@
       <c r="H31">
         <v>39.1</v>
       </c>
+      <c r="J31">
+        <v>8.609999999999999</v>
+      </c>
       <c r="L31">
-        <v>28.447590297657</v>
+        <v>28.45496160547599</v>
       </c>
       <c r="N31">
         <v>14.48535819563911</v>
@@ -2224,6 +2397,9 @@
       </c>
       <c r="U31">
         <v>0.5353455265318441</v>
+      </c>
+      <c r="V31">
+        <v>7.371307818991098</v>
       </c>
       <c r="Z31">
         <v>556.453310874829</v>
@@ -2248,8 +2424,11 @@
       <c r="H32">
         <v>50</v>
       </c>
+      <c r="J32">
+        <v>9.119999999999999</v>
+      </c>
       <c r="L32">
-        <v>7.224941125858438</v>
+        <v>7.226190035174804</v>
       </c>
       <c r="N32">
         <v>3.922555200532898</v>
@@ -2271,6 +2450,9 @@
       </c>
       <c r="U32">
         <v>0.0425184726701672</v>
+      </c>
+      <c r="V32">
+        <v>1.248909316366126</v>
       </c>
       <c r="Z32">
         <v>796.220654805769</v>
@@ -2295,8 +2477,11 @@
       <c r="H33">
         <v>55.5</v>
       </c>
+      <c r="J33">
+        <v>9.050000000000001</v>
+      </c>
       <c r="L33">
-        <v>7.236286267985585</v>
+        <v>7.237561726344408</v>
       </c>
       <c r="N33">
         <v>3.968495482055518</v>
@@ -2318,6 +2503,9 @@
       </c>
       <c r="U33">
         <v>0.0401526409076609</v>
+      </c>
+      <c r="V33">
+        <v>1.275458358822187</v>
       </c>
       <c r="Z33">
         <v>798.3893041372776</v>
@@ -2342,8 +2530,11 @@
       <c r="H34">
         <v>38</v>
       </c>
+      <c r="J34">
+        <v>8.029999999999999</v>
+      </c>
       <c r="L34">
-        <v>12.65630421083764</v>
+        <v>12.66037197087645</v>
       </c>
       <c r="N34">
         <v>6.796407071336819</v>
@@ -2365,6 +2556,9 @@
       </c>
       <c r="U34">
         <v>0.0758677487256479</v>
+      </c>
+      <c r="V34">
+        <v>4.067760038803926</v>
       </c>
       <c r="Z34">
         <v>372.6023791978103</v>
@@ -2389,8 +2583,11 @@
       <c r="H35">
         <v>67.5</v>
       </c>
+      <c r="J35">
+        <v>9.41</v>
+      </c>
       <c r="L35">
-        <v>5.57301837633096</v>
+        <v>5.5735273047085</v>
       </c>
       <c r="N35">
         <v>2.436474704030302</v>
@@ -2412,6 +2609,9 @@
       </c>
       <c r="U35">
         <v>0.0224383157323975</v>
+      </c>
+      <c r="V35">
+        <v>0.5089283775393745</v>
       </c>
       <c r="Z35">
         <v>176.4238340877987</v>
@@ -2436,8 +2636,11 @@
       <c r="H36">
         <v>75</v>
       </c>
+      <c r="J36">
+        <v>6.79</v>
+      </c>
       <c r="L36">
-        <v>27.57355782226824</v>
+        <v>27.58418000919817</v>
       </c>
       <c r="N36">
         <v>13.50761111605776</v>
@@ -2462,6 +2665,9 @@
       </c>
       <c r="U36">
         <v>0.5060475775161579</v>
+      </c>
+      <c r="V36">
+        <v>10.62218692992467</v>
       </c>
       <c r="Z36">
         <v>523.6814401515949</v>
@@ -2486,8 +2692,11 @@
       <c r="H37">
         <v>57.7</v>
       </c>
+      <c r="J37">
+        <v>9.08</v>
+      </c>
       <c r="L37">
-        <v>3.006819584416952</v>
+        <v>3.006830238733608</v>
       </c>
       <c r="N37">
         <v>2.40435212724408</v>
@@ -2509,6 +2718,9 @@
       </c>
       <c r="U37">
         <v>0.0683073177094656</v>
+      </c>
+      <c r="V37">
+        <v>0.0106543166560146</v>
       </c>
       <c r="Z37">
         <v>366.022739235709</v>
@@ -2533,8 +2745,11 @@
       <c r="H38">
         <v>46.9</v>
       </c>
+      <c r="J38">
+        <v>9.32</v>
+      </c>
       <c r="L38">
-        <v>7.426394862496641</v>
+        <v>7.426996898122183</v>
       </c>
       <c r="N38">
         <v>3.728702102226429</v>
@@ -2556,6 +2771,9 @@
       </c>
       <c r="U38">
         <v>0.055841302563027</v>
+      </c>
+      <c r="V38">
+        <v>0.6020356255421137</v>
       </c>
       <c r="Z38">
         <v>400.542162332877</v>
@@ -2580,8 +2798,11 @@
       <c r="H39">
         <v>45.7</v>
       </c>
+      <c r="J39">
+        <v>8.949999999999999</v>
+      </c>
       <c r="L39">
-        <v>8.346598766100309</v>
+        <v>8.347036571362464</v>
       </c>
       <c r="N39">
         <v>4.60926336406425</v>
@@ -2606,6 +2827,9 @@
       </c>
       <c r="U39">
         <v>0.0482962174826015</v>
+      </c>
+      <c r="V39">
+        <v>0.4378052621547591</v>
       </c>
       <c r="Z39">
         <v>127.6186967049163</v>
@@ -2630,8 +2854,11 @@
       <c r="H40">
         <v>59.6</v>
       </c>
+      <c r="J40">
+        <v>8.24</v>
+      </c>
       <c r="L40">
-        <v>9.432322672258429</v>
+        <v>9.433394912505291</v>
       </c>
       <c r="N40">
         <v>4.688011436739535</v>
@@ -2656,6 +2883,9 @@
       </c>
       <c r="U40">
         <v>0.1093576958588992</v>
+      </c>
+      <c r="V40">
+        <v>1.072240246861447</v>
       </c>
       <c r="Z40">
         <v>693.9204126750184</v>
@@ -2680,8 +2910,11 @@
       <c r="H41">
         <v>72</v>
       </c>
+      <c r="J41">
+        <v>9.369999999999999</v>
+      </c>
       <c r="L41">
-        <v>11.93500807938937</v>
+        <v>11.93502240627209</v>
       </c>
       <c r="N41">
         <v>5.934935666382729</v>
@@ -2703,6 +2936,9 @@
       </c>
       <c r="U41">
         <v>0.0406309225720811</v>
+      </c>
+      <c r="V41">
+        <v>0.0143268827208399</v>
       </c>
       <c r="Z41">
         <v>1274.971049584167</v>
@@ -2727,8 +2963,11 @@
       <c r="H42">
         <v>58.8</v>
       </c>
+      <c r="J42">
+        <v>9.24</v>
+      </c>
       <c r="L42">
-        <v>9.006946365449402</v>
+        <v>9.006959896781083</v>
       </c>
       <c r="N42">
         <v>4.209311542016799</v>
@@ -2750,6 +2989,9 @@
       </c>
       <c r="U42">
         <v>0.0421834197394771</v>
+      </c>
+      <c r="V42">
+        <v>0.0135313316822643</v>
       </c>
       <c r="Z42">
         <v>599.4578376671228</v>
@@ -2774,8 +3016,11 @@
       <c r="H43">
         <v>58.5</v>
       </c>
+      <c r="J43">
+        <v>9.15</v>
+      </c>
       <c r="L43">
-        <v>7.826277218037141</v>
+        <v>7.826290647418663</v>
       </c>
       <c r="N43">
         <v>4.128001460127764</v>
@@ -2797,6 +3042,9 @@
       </c>
       <c r="U43">
         <v>0.0408841305120682</v>
+      </c>
+      <c r="V43">
+        <v>0.0134293815224834</v>
       </c>
       <c r="Z43">
         <v>597.7787135487946</v>

</xml_diff>